<commit_message>
model 36h fixed continuous and rolling
</commit_message>
<xml_diff>
--- a/Cost results_NEDdata1703.xlsx
+++ b/Cost results_NEDdata1703.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tenneteu-my.sharepoint.com/personal/laura_linuesa-domenech_tennet_eu/Documents/Thesis/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="757" documentId="8_{BA558C3F-E59C-4F04-9D2E-8441DAA40C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AE06F12-5C49-4232-ABF6-147A8239056A}"/>
+  <xr:revisionPtr revIDLastSave="765" documentId="8_{BA558C3F-E59C-4F04-9D2E-8441DAA40C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EE8D4B6-ED36-436F-A78A-063338D15460}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{4AE1EDD8-8ACF-4AF9-86A6-B0088C54F040}"/>
   </bookViews>
@@ -1434,7 +1434,7 @@
         <v>59</v>
       </c>
       <c r="F4" s="8">
-        <v>109.44068339440538</v>
+        <v>108.76824513184334</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -1442,16 +1442,16 @@
         <v>48</v>
       </c>
       <c r="B5" s="8">
-        <v>2811258631.9539056</v>
+        <v>2811043012.3559942</v>
       </c>
       <c r="C5" s="8">
-        <v>93708621.065130189</v>
+        <v>93701433.745199814</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>57</v>
       </c>
       <c r="F5" s="8">
-        <v>15130.4496253816</v>
+        <v>18892.793002505448</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -1459,10 +1459,10 @@
         <v>49</v>
       </c>
       <c r="B6" s="8">
-        <v>359967997.883524</v>
+        <v>359629075.69536591</v>
       </c>
       <c r="C6" s="8">
-        <v>11998933.262784133</v>
+        <v>11987635.856512196</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -1470,10 +1470,10 @@
         <v>50</v>
       </c>
       <c r="B7" s="8">
-        <v>2451290634.0703816</v>
+        <v>2451413936.6606283</v>
       </c>
       <c r="C7" s="8">
-        <v>81709687.802346051</v>
+        <v>81713797.888687611</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -1507,16 +1507,16 @@
         <v>5</v>
       </c>
       <c r="B11" s="8">
-        <v>3975223.6106515261</v>
+        <v>3982876.9199949773</v>
       </c>
       <c r="C11" s="8">
-        <v>447388210.71222073</v>
+        <v>445596795.14286435</v>
       </c>
       <c r="D11" s="8">
-        <v>112.54416217328092</v>
+        <v>111.87812329973437</v>
       </c>
       <c r="E11" s="8">
-        <v>14912940.357074024</v>
+        <v>14853226.504762145</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
@@ -1524,16 +1524,16 @@
         <v>31</v>
       </c>
       <c r="B12" s="8">
-        <v>1634705.9184592848</v>
+        <v>1628038.5824713197</v>
       </c>
       <c r="C12" s="8">
-        <v>239295579.20617732</v>
+        <v>236128137.90835813</v>
       </c>
       <c r="D12" s="8">
-        <v>146.38448206740091</v>
+        <v>145.03841644214711</v>
       </c>
       <c r="E12" s="8">
-        <v>7976519.3068725774</v>
+        <v>7870937.9302786039</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
@@ -1541,16 +1541,16 @@
         <v>6</v>
       </c>
       <c r="B13" s="8">
-        <v>732898.7739149027</v>
+        <v>732664.54331873974</v>
       </c>
       <c r="C13" s="8">
-        <v>138488149.42056879</v>
+        <v>134703014.83114436</v>
       </c>
       <c r="D13" s="8">
-        <v>188.95945026734174</v>
+        <v>183.85360129614313</v>
       </c>
       <c r="E13" s="8">
-        <v>4616271.6473522931</v>
+        <v>4490100.4943714784</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
@@ -1561,13 +1561,13 @@
         <v>478312.56544999999</v>
       </c>
       <c r="C14" s="8">
-        <v>39041979.760479055</v>
+        <v>38925180.534927145</v>
       </c>
       <c r="D14" s="8">
-        <v>81.624407512163245</v>
+        <v>81.380217344501602</v>
       </c>
       <c r="E14" s="8">
-        <v>1301399.3253493018</v>
+        <v>1297506.0178309048</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
@@ -1575,16 +1575,16 @@
         <v>7</v>
       </c>
       <c r="B15" s="8">
-        <v>2767691.1981246169</v>
+        <v>2763928.8547474938</v>
       </c>
       <c r="C15" s="8">
-        <v>185194415.22348258</v>
+        <v>187279850.58477989</v>
       </c>
       <c r="D15" s="8">
-        <v>66.912961731052235</v>
+        <v>67.758564140714597</v>
       </c>
       <c r="E15" s="8">
-        <v>6173147.1741160862</v>
+        <v>6242661.6861593295</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -1592,13 +1592,13 @@
         <v>8</v>
       </c>
       <c r="B16" s="8">
-        <v>9588832.0666003302</v>
+        <v>9585821.4659825303</v>
       </c>
       <c r="C16" s="8">
-        <v>1049408334.3229285</v>
+        <v>1042632979.0020738</v>
       </c>
       <c r="E16" s="8">
-        <v>34980277.810764283</v>
+        <v>34754432.633402459</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1632,16 +1632,16 @@
         <v>5</v>
       </c>
       <c r="B20" s="8">
-        <v>452379607.22834575</v>
+        <v>448566332.41025943</v>
       </c>
       <c r="C20" s="8">
-        <v>4113223.6106515257</v>
+        <v>4120876.9199949773</v>
       </c>
       <c r="D20" s="8">
-        <v>4661510.7483778223</v>
+        <v>4634643.3879737807</v>
       </c>
       <c r="E20" s="8">
-        <v>15079320.240944859</v>
+        <v>14952211.080341982</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1649,16 +1649,16 @@
         <v>31</v>
       </c>
       <c r="B21" s="8">
-        <v>246771741.03197482</v>
+        <v>243394966.75958812</v>
       </c>
       <c r="C21" s="8">
-        <v>1724646.3557952398</v>
+        <v>1717754.4742361107</v>
       </c>
       <c r="D21" s="8">
-        <v>2615025.7866429016</v>
+        <v>2652099.8573610727</v>
       </c>
       <c r="E21" s="8">
-        <v>8225724.7010658272</v>
+        <v>8113165.5586529374</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -1666,16 +1666,16 @@
         <v>6</v>
       </c>
       <c r="B22" s="8">
-        <v>137966369.87963834</v>
+        <v>137343384.36182228</v>
       </c>
       <c r="C22" s="8">
-        <v>760764.41212537326</v>
+        <v>761478.05516458466</v>
       </c>
       <c r="D22" s="8">
-        <v>2073773.9403398721</v>
+        <v>2061822.8216769036</v>
       </c>
       <c r="E22" s="8">
-        <v>4598878.9959879452</v>
+        <v>4578112.8120607426</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -1683,7 +1683,7 @@
         <v>32</v>
       </c>
       <c r="B23" s="8">
-        <v>40147138.037544556</v>
+        <v>40159749.943126753</v>
       </c>
       <c r="C23" s="8">
         <v>492550.3836</v>
@@ -1692,7 +1692,7 @@
         <v>492550.3836</v>
       </c>
       <c r="E23" s="8">
-        <v>1338237.9345848185</v>
+        <v>1338658.3314375584</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -1700,16 +1700,16 @@
         <v>7</v>
       </c>
       <c r="B24" s="8">
-        <v>171491152.3333112</v>
+        <v>169561145.75714132</v>
       </c>
       <c r="C24" s="8">
-        <v>2812589.9173202403</v>
+        <v>2808100.0982027063</v>
       </c>
       <c r="D24" s="8">
-        <v>5203603.0745604774</v>
+        <v>5131115.2235797457</v>
       </c>
       <c r="E24" s="8">
-        <v>5716371.7444437062</v>
+        <v>5652038.1919047106</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -1717,10 +1717,10 @@
         <v>12</v>
       </c>
       <c r="B25" s="8">
-        <v>1048756008.5108147</v>
+        <v>1039025579.2319379</v>
       </c>
       <c r="E25" s="8">
-        <v>34958533.617027156</v>
+        <v>34634185.974397928</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -1746,10 +1746,10 @@
         <v>5</v>
       </c>
       <c r="B29" s="8">
-        <v>119256708.31954573</v>
+        <v>119486307.59984931</v>
       </c>
       <c r="C29" s="8">
-        <v>3975223.6106515243</v>
+        <v>3982876.9199949773</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -1757,10 +1757,10 @@
         <v>31</v>
       </c>
       <c r="B30" s="8">
-        <v>130776473.47674279</v>
+        <v>130243086.59770559</v>
       </c>
       <c r="C30" s="8">
-        <v>4359215.7825580928</v>
+        <v>4341436.2199235195</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -1768,10 +1768,10 @@
         <v>6</v>
       </c>
       <c r="B31" s="8">
-        <v>109934816.08723547</v>
+        <v>109899681.497811</v>
       </c>
       <c r="C31" s="8">
-        <v>3664493.8695745156</v>
+        <v>3663322.7165937</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -1801,10 +1801,10 @@
         <v>14</v>
       </c>
       <c r="B34" s="8">
-        <v>359967997.883524</v>
+        <v>359629075.69536591</v>
       </c>
       <c r="C34" s="8">
-        <v>11998933.262784133</v>
+        <v>11987635.856512196</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -1812,7 +1812,7 @@
         <v>15</v>
       </c>
       <c r="B35" s="8">
-        <v>516453.36855598853</v>
+        <v>515967.11003639299</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -1838,10 +1838,10 @@
         <v>5</v>
       </c>
       <c r="B39" s="8">
-        <v>333122898.90880001</v>
+        <v>329080024.81041014</v>
       </c>
       <c r="C39" s="8">
-        <v>11104096.630293334</v>
+        <v>10969334.160347005</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
@@ -1849,10 +1849,10 @@
         <v>31</v>
       </c>
       <c r="B40" s="8">
-        <v>115995267.55523203</v>
+        <v>113151880.16188253</v>
       </c>
       <c r="C40" s="8">
-        <v>3866508.9185077343</v>
+        <v>3771729.3387294179</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="12.4" customHeight="1" x14ac:dyDescent="0.35">
@@ -1860,10 +1860,10 @@
         <v>6</v>
       </c>
       <c r="B41" s="8">
-        <v>28031553.792402878</v>
+        <v>27443702.864011273</v>
       </c>
       <c r="C41" s="8">
-        <v>934385.12641342927</v>
+        <v>914790.09546704241</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -1871,10 +1871,10 @@
         <v>32</v>
       </c>
       <c r="B42" s="8">
-        <v>40147138.037544556</v>
+        <v>40159749.943126753</v>
       </c>
       <c r="C42" s="8">
-        <v>1338237.9345848185</v>
+        <v>1338658.3314375584</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1882,10 +1882,10 @@
         <v>7</v>
       </c>
       <c r="B43" s="8">
-        <v>171491152.3333112</v>
+        <v>169561145.75714132</v>
       </c>
       <c r="C43" s="8">
-        <v>5716371.7444437062</v>
+        <v>5652038.1919047106</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
@@ -1893,10 +1893,10 @@
         <v>17</v>
       </c>
       <c r="B44" s="8">
-        <v>688788010.62729073</v>
+        <v>679396503.53657198</v>
       </c>
       <c r="C44" s="8">
-        <v>22959600.354243021</v>
+        <v>22646550.117885731</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
@@ -1921,10 +1921,10 @@
         <v>40</v>
       </c>
       <c r="B48" s="8">
-        <v>200833.08239874837</v>
+        <v>204599.28922255122</v>
       </c>
       <c r="C48" s="8">
-        <v>6694.4360799582792</v>
+        <v>6819.9763074183738</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
@@ -1932,10 +1932,10 @@
         <v>41</v>
       </c>
       <c r="B49" s="8">
-        <v>248601.76273549208</v>
+        <v>253251.40078956936</v>
       </c>
       <c r="C49" s="8">
-        <v>8286.7254245164022</v>
+        <v>8441.7133596523126</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
@@ -1943,7 +1943,7 @@
         <v>19</v>
       </c>
       <c r="B50" s="8">
-        <v>151.25461735672505</v>
+        <v>147.37183863930306</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>51</v>
@@ -1954,7 +1954,7 @@
         <v>20</v>
       </c>
       <c r="B51" s="8">
-        <v>82.707146935248772</v>
+        <v>82.831418924411182</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
@@ -1962,10 +1962,10 @@
         <v>21</v>
       </c>
       <c r="B52" s="8">
-        <v>30376931.030794315</v>
+        <v>30152173.437021919</v>
       </c>
       <c r="C52" s="8">
-        <v>1012564.3676931438</v>
+        <v>1005072.4479007307</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
@@ -1973,10 +1973,10 @@
         <v>22</v>
       </c>
       <c r="B53" s="8">
-        <v>20561142.518926196</v>
+        <v>20977172.871994779</v>
       </c>
       <c r="C53" s="8">
-        <v>685371.41729753988</v>
+        <v>699239.09573315934</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
@@ -1984,10 +1984,10 @@
         <v>23</v>
       </c>
       <c r="B54" s="8">
-        <v>9815788.5118681192</v>
+        <v>9175000.5650271401</v>
       </c>
       <c r="C54" s="8">
-        <v>327192.95039560396</v>
+        <v>305833.35216757131</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
@@ -1995,10 +1995,10 @@
         <v>60</v>
       </c>
       <c r="B55" s="8">
-        <v>47768.68033674371</v>
+        <v>48058.394437018149</v>
       </c>
       <c r="C55" s="8">
-        <v>1592.2893445581237</v>
+        <v>1601.9464812339384</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
@@ -2006,7 +2006,7 @@
         <v>61</v>
       </c>
       <c r="B56" s="8">
-        <v>0</v>
+        <v>593.71712999999988</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
@@ -2036,10 +2036,10 @@
         <v>5</v>
       </c>
       <c r="B60" s="8">
-        <v>3975223.6106515261</v>
+        <v>3982876.9199949773</v>
       </c>
       <c r="C60" s="8">
-        <v>3975223.6106515261</v>
+        <v>3982876.9199949773</v>
       </c>
       <c r="D60" s="8">
         <v>0</v>
@@ -2050,13 +2050,13 @@
         <v>31</v>
       </c>
       <c r="B61" s="8">
-        <v>1634705.9184592848</v>
+        <v>1628038.5824713197</v>
       </c>
       <c r="C61" s="8">
-        <v>1634705.9184592848</v>
+        <v>1628038.5824713197</v>
       </c>
       <c r="D61" s="8">
-        <v>2.8421709430404007E-14</v>
+        <v>1.1368683772161603E-13</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
@@ -2064,10 +2064,10 @@
         <v>6</v>
       </c>
       <c r="B62" s="8">
-        <v>732898.7739149027</v>
+        <v>732664.54331873974</v>
       </c>
       <c r="C62" s="8">
-        <v>732898.7739149027</v>
+        <v>732664.54331873974</v>
       </c>
       <c r="D62" s="8">
         <v>4.5474735088646412E-13</v>
@@ -2092,10 +2092,10 @@
         <v>7</v>
       </c>
       <c r="B64" s="8">
-        <v>2767691.1981246169</v>
+        <v>2763928.8547474938</v>
       </c>
       <c r="C64" s="8">
-        <v>2767691.1981246169</v>
+        <v>2763928.8547474938</v>
       </c>
       <c r="D64" s="8">
         <v>0</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="C65" s="8">
         <f>SUM(C60:C64)</f>
-        <v>9588832.0666003302</v>
+        <v>9585821.4659825303</v>
       </c>
     </row>
   </sheetData>
@@ -2147,11 +2147,11 @@
       </c>
       <c r="C2" s="8">
         <f>Fixed!C34</f>
-        <v>11998933.262784133</v>
+        <v>11987635.856512196</v>
       </c>
       <c r="D2" s="15">
         <f>(C2-B2)/B2</f>
-        <v>5.5480808607984884E-3</v>
+        <v>4.6013229326845968E-3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="C3" s="8">
         <f>Fixed!C54</f>
-        <v>327192.95039560396</v>
+        <v>305833.35216757131</v>
       </c>
       <c r="D3" s="14">
         <f>(C3-B3)/B3</f>
-        <v>-2.9641375007708297E-2</v>
+        <v>-9.2987698153978685E-2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -2181,11 +2181,11 @@
       </c>
       <c r="C4" s="8">
         <f>Fixed!C7</f>
-        <v>81709687.802346051</v>
+        <v>81713797.888687611</v>
       </c>
       <c r="D4" s="15">
         <f t="shared" ref="D4" si="0">(C4-B4)/B4</f>
-        <v>-7.2891629337627436E-4</v>
+        <v>-6.7865186888608044E-4</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="C6" s="8">
         <f>Fixed!E20</f>
-        <v>15079320.240944859</v>
+        <v>14952211.080341982</v>
       </c>
       <c r="D6" s="14">
         <f>(C6-B6)/B6</f>
-        <v>0.12868781475576935</v>
+        <v>0.11917368822858368</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -2223,11 +2223,11 @@
       </c>
       <c r="C7" s="8">
         <f>Fixed!E21</f>
-        <v>8225724.7010658272</v>
+        <v>8113165.5586529374</v>
       </c>
       <c r="D7" s="14">
         <f>(C7-B7)/B7</f>
-        <v>0.10327119522246568</v>
+        <v>8.8174256764630615E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -2240,11 +2240,11 @@
       </c>
       <c r="C8" s="8">
         <f>Fixed!E22</f>
-        <v>4598878.9959879452</v>
+        <v>4578112.8120607426</v>
       </c>
       <c r="D8" s="14">
         <f>(C8-B8)/B8</f>
-        <v>7.7066834289878039E-2</v>
+        <v>7.2203351688516701E-2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -2257,11 +2257,11 @@
       </c>
       <c r="C9" s="8">
         <f>Fixed!E23</f>
-        <v>1338237.9345848185</v>
+        <v>1338658.3314375584</v>
       </c>
       <c r="D9" s="14">
         <f>(C9-B9)/B9</f>
-        <v>0.1918277563045476</v>
+        <v>0.19220215955886416</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -2274,11 +2274,11 @@
       </c>
       <c r="C10" s="8">
         <f>Fixed!E24</f>
-        <v>5716371.7444437062</v>
+        <v>5652038.1919047106</v>
       </c>
       <c r="D10" s="14">
         <f>(C10-B10)/B10</f>
-        <v>0.21688164644016281</v>
+        <v>0.20318654002741215</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">

</xml_diff>